<commit_message>
Templates de condomínio atualizados e formato de célula ajustado
- Novos templates Amplo (com aba Auxiliar e linha de exemplo) e
  Tradicional (ordem das primeiras coberturas alterada).
- Formato dos condomínios pelos exemplos novos: opção desmarcada e
  cobertura não contratada '<IGNORE>' (antes 'Não'/vazio); indenização do
  condomínio continua 'Sim'/'Não'; valores como número.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETeciituSBa5wphWUasW8C
</commit_message>
<xml_diff>
--- a/.claude/skills/gerador-massas-seguros/templates/template_condominio_amplo.xlsx
+++ b/.claude/skills/gerador-massas-seguros/templates/template_condominio_amplo.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb35177745223ee1/Área de Trabalho/TEMPLATES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="8_{F0EDC613-234C-410C-B7C7-5693FD68759D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9C14DE4-D8F3-4F13-9B1C-E3CA1DCBFA7C}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{85FCB343-C9DD-4353-81A7-D8F49E45ACB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DD1C27E-6F33-48C3-A62E-D1292AF8AF75}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D1778361-77A0-49C1-A6FF-9F11D3ACD25C}"/>
   </bookViews>
   <sheets>
     <sheet name="Cotação" sheetId="1" r:id="rId1"/>
+    <sheet name="Auxiliar" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188483" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="83">
   <si>
     <t>Dados CORRETOR</t>
   </si>
@@ -260,17 +261,46 @@
     <t>COI</t>
   </si>
   <si>
-    <t>Espaco informatica</t>
-  </si>
-  <si>
-    <t>Sicredi</t>
+    <t xml:space="preserve"> Tipo de Condomínio</t>
+  </si>
+  <si>
+    <t>Tipo de Construção</t>
+  </si>
+  <si>
+    <t>Objeto Segurado</t>
+  </si>
+  <si>
+    <t>Assistência 24h INPUT</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>6 ou mais</t>
+  </si>
+  <si>
+    <t>Não informado</t>
+  </si>
+  <si>
+    <t>Período Indenitário" Perda Ou Pagamento de Aluguel a Terceiros</t>
+  </si>
+  <si>
+    <t>&lt;IGNORE&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="00000000000000"/>
+    <numFmt numFmtId="165" formatCode="00000000"/>
+  </numFmts>
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,11 +319,13 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFF3F3F3"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -316,10 +348,25 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="16">
@@ -476,10 +523,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -510,12 +558,24 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -536,7 +596,8 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -873,19 +934,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DB94AD-DD93-48A3-87B2-8FB065BB5A7F}">
-  <dimension ref="A1:AY10"/>
+  <dimension ref="A1:AY33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" customWidth="1"/>
     <col min="5" max="5" width="50.28515625" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="58.7109375" customWidth="1"/>
     <col min="9" max="9" width="33" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="60.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="29.42578125" bestFit="1" customWidth="1"/>
@@ -893,7 +954,7 @@
     <col min="15" max="15" width="77.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="78.28515625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="82.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="76.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="77.28515625" customWidth="1"/>
     <col min="19" max="19" width="82.7109375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="41.7109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="40.7109375" bestFit="1" customWidth="1"/>
@@ -923,18 +984,18 @@
   <sheetData>
     <row r="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="19" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
       <c r="J1" s="2" t="s">
         <v>2</v>
       </c>
@@ -947,23 +1008,23 @@
       <c r="M1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="N1" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
       <c r="S1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="T1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
       <c r="Y1" s="12" t="s">
         <v>9</v>
       </c>
@@ -978,23 +1039,23 @@
       <c r="AH1" s="12"/>
       <c r="AI1" s="12"/>
       <c r="AJ1" s="12"/>
-      <c r="AK1" s="22" t="s">
+      <c r="AK1" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="AL1" s="22"/>
-      <c r="AM1" s="22"/>
-      <c r="AN1" s="22"/>
-      <c r="AO1" s="22"/>
-      <c r="AP1" s="22"/>
-      <c r="AQ1" s="22"/>
-      <c r="AR1" s="22"/>
-      <c r="AS1" s="16"/>
-      <c r="AT1" s="16"/>
-      <c r="AU1" s="16"/>
-      <c r="AV1" s="16"/>
-      <c r="AW1" s="16"/>
-      <c r="AX1" s="16"/>
-      <c r="AY1" s="16"/>
+      <c r="AL1" s="28"/>
+      <c r="AM1" s="28"/>
+      <c r="AN1" s="28"/>
+      <c r="AO1" s="28"/>
+      <c r="AP1" s="28"/>
+      <c r="AQ1" s="28"/>
+      <c r="AR1" s="28"/>
+      <c r="AS1" s="22"/>
+      <c r="AT1" s="22"/>
+      <c r="AU1" s="22"/>
+      <c r="AV1" s="22"/>
+      <c r="AW1" s="22"/>
+      <c r="AX1" s="22"/>
+      <c r="AY1" s="22"/>
     </row>
     <row r="2" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
@@ -1009,7 +1070,7 @@
       <c r="D2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="11" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="9" t="s">
@@ -1033,7 +1094,7 @@
       <c r="L2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="11" t="s">
         <v>23</v>
       </c>
       <c r="N2" s="9" t="s">
@@ -1129,10 +1190,10 @@
       <c r="AR2" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="AS2" s="15"/>
-      <c r="AT2" s="15"/>
-      <c r="AU2" s="15"/>
-      <c r="AV2" s="15"/>
+      <c r="AS2" s="14"/>
+      <c r="AT2" s="14"/>
+      <c r="AU2" s="14"/>
+      <c r="AV2" s="14"/>
     </row>
     <row r="3" spans="1:51" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1141,14 +1202,14 @@
       <c r="B3" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="14">
-        <v>42907871865</v>
-      </c>
-      <c r="D3" s="14">
-        <v>6417050</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>55</v>
+      <c r="C3" s="15">
+        <v>72066486000171</v>
+      </c>
+      <c r="D3" s="16">
+        <v>8040770</v>
+      </c>
+      <c r="E3" t="s">
+        <v>59</v>
       </c>
       <c r="F3" s="13" t="s">
         <v>63</v>
@@ -1157,67 +1218,649 @@
         <v>66</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+      <c r="I3" s="19">
+        <v>1000000</v>
+      </c>
+      <c r="J3" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+      <c r="N3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="O3" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="P3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="R3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="S3" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="T3" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="U3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="W3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="X3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y3" s="19">
+        <v>50000</v>
+      </c>
+      <c r="Z3" s="19">
+        <v>35000</v>
+      </c>
+      <c r="AA3" s="19">
+        <v>75000</v>
+      </c>
+      <c r="AB3" s="19">
+        <v>35000</v>
+      </c>
+      <c r="AC3" s="21">
+        <v>6</v>
+      </c>
+      <c r="AD3" s="19">
+        <v>10000</v>
+      </c>
+      <c r="AE3" s="19">
+        <v>10000</v>
+      </c>
+      <c r="AF3" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>82</v>
+      </c>
+      <c r="AH3" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AI3" s="19">
+        <v>3000</v>
+      </c>
+      <c r="AJ3" s="19">
+        <v>35000</v>
+      </c>
+      <c r="AK3" s="19">
+        <v>5000</v>
+      </c>
+      <c r="AL3" s="21">
+        <v>10</v>
+      </c>
+      <c r="AM3" s="19">
+        <v>5000</v>
+      </c>
+      <c r="AN3" s="19">
+        <v>5000</v>
+      </c>
+      <c r="AO3" s="19">
+        <v>5000</v>
+      </c>
+      <c r="AP3" s="19">
+        <v>1000</v>
+      </c>
+      <c r="AQ3" s="19"/>
+      <c r="AR3" s="19">
+        <v>3000</v>
       </c>
     </row>
     <row r="4" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>68</v>
-      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="16"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="19"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20"/>
+      <c r="X4" s="20"/>
+      <c r="Y4" s="19"/>
+      <c r="Z4" s="19"/>
+      <c r="AA4" s="19"/>
+      <c r="AB4" s="19"/>
+      <c r="AC4" s="21"/>
+      <c r="AD4" s="19"/>
+      <c r="AE4" s="19"/>
+      <c r="AF4" s="19"/>
+      <c r="AG4" s="19"/>
+      <c r="AH4" s="19"/>
+      <c r="AI4" s="19"/>
+      <c r="AJ4" s="19"/>
+      <c r="AK4" s="19"/>
+      <c r="AL4" s="21"/>
+      <c r="AM4" s="19"/>
+      <c r="AN4" s="19"/>
+      <c r="AO4" s="19"/>
+      <c r="AP4" s="19"/>
+      <c r="AQ4" s="19"/>
+      <c r="AR4" s="19"/>
     </row>
     <row r="5" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>69</v>
-      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="16"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="19"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20"/>
+      <c r="X5" s="20"/>
+      <c r="Y5" s="19"/>
+      <c r="Z5" s="19"/>
+      <c r="AA5" s="19"/>
+      <c r="AB5" s="19"/>
+      <c r="AC5" s="21"/>
+      <c r="AD5" s="19"/>
+      <c r="AE5" s="19"/>
+      <c r="AF5" s="19"/>
+      <c r="AH5" s="19"/>
+      <c r="AI5" s="19"/>
+      <c r="AJ5" s="19"/>
+      <c r="AK5" s="19"/>
+      <c r="AL5" s="21"/>
+      <c r="AM5" s="19"/>
+      <c r="AN5" s="19"/>
+      <c r="AO5" s="19"/>
+      <c r="AP5" s="19"/>
+      <c r="AQ5" s="19"/>
+      <c r="AR5" s="19"/>
     </row>
     <row r="6" spans="1:51" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="13" t="s">
-        <v>58</v>
-      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="19"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
+      <c r="U6" s="20"/>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20"/>
+      <c r="X6" s="20"/>
+      <c r="Y6" s="19"/>
+      <c r="Z6" s="19"/>
+      <c r="AA6" s="19"/>
+      <c r="AB6" s="19"/>
+      <c r="AC6" s="21"/>
+      <c r="AD6" s="19"/>
+      <c r="AE6" s="19"/>
+      <c r="AF6" s="19"/>
+      <c r="AH6" s="19"/>
+      <c r="AI6" s="19"/>
+      <c r="AJ6" s="19"/>
+      <c r="AK6" s="19"/>
+      <c r="AL6" s="21"/>
+      <c r="AM6" s="19"/>
+      <c r="AN6" s="19"/>
+      <c r="AO6" s="19"/>
+      <c r="AP6" s="19"/>
+      <c r="AQ6" s="19"/>
+      <c r="AR6" s="19"/>
     </row>
     <row r="7" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="E7" s="13" t="s">
-        <v>59</v>
-      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="19"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
+      <c r="X7" s="20"/>
+      <c r="Y7" s="19"/>
+      <c r="Z7" s="19"/>
+      <c r="AA7" s="19"/>
+      <c r="AB7" s="19"/>
+      <c r="AC7" s="21"/>
+      <c r="AD7" s="19"/>
+      <c r="AE7" s="19"/>
+      <c r="AF7" s="19"/>
+      <c r="AH7" s="19"/>
+      <c r="AI7" s="19"/>
+      <c r="AJ7" s="19"/>
+      <c r="AK7" s="19"/>
+      <c r="AL7" s="21"/>
+      <c r="AM7" s="19"/>
+      <c r="AN7" s="19"/>
+      <c r="AO7" s="19"/>
+      <c r="AP7" s="19"/>
+      <c r="AQ7" s="19"/>
+      <c r="AR7" s="19"/>
     </row>
     <row r="8" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="E8" s="13" t="s">
-        <v>60</v>
-      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="19"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20"/>
+      <c r="X8" s="20"/>
+      <c r="Y8" s="19"/>
+      <c r="Z8" s="19"/>
+      <c r="AA8" s="19"/>
+      <c r="AB8" s="19"/>
+      <c r="AC8" s="21"/>
+      <c r="AD8" s="19"/>
+      <c r="AE8" s="19"/>
+      <c r="AF8" s="19"/>
+      <c r="AH8" s="19"/>
+      <c r="AI8" s="19"/>
+      <c r="AJ8" s="19"/>
+      <c r="AK8" s="19"/>
+      <c r="AL8" s="21"/>
+      <c r="AM8" s="19"/>
+      <c r="AN8" s="19"/>
+      <c r="AO8" s="19"/>
+      <c r="AP8" s="19"/>
+      <c r="AQ8" s="19"/>
+      <c r="AR8" s="19"/>
     </row>
     <row r="9" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="E9" s="13" t="s">
-        <v>61</v>
-      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="19"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
+      <c r="T9" s="20"/>
+      <c r="U9" s="20"/>
+      <c r="V9" s="20"/>
+      <c r="W9" s="20"/>
+      <c r="X9" s="20"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="19"/>
+      <c r="AA9" s="19"/>
+      <c r="AB9" s="19"/>
+      <c r="AC9" s="21"/>
+      <c r="AD9" s="19"/>
+      <c r="AE9" s="19"/>
+      <c r="AF9" s="19"/>
+      <c r="AH9" s="19"/>
+      <c r="AI9" s="19"/>
+      <c r="AJ9" s="19"/>
+      <c r="AK9" s="19"/>
+      <c r="AL9" s="21"/>
+      <c r="AM9" s="19"/>
+      <c r="AN9" s="19"/>
+      <c r="AO9" s="19"/>
+      <c r="AP9" s="19"/>
+      <c r="AQ9" s="19"/>
+      <c r="AR9" s="19"/>
     </row>
     <row r="10" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="E10" s="13" t="s">
-        <v>62</v>
-      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="19"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="20"/>
+      <c r="S10" s="20"/>
+      <c r="T10" s="20"/>
+      <c r="U10" s="20"/>
+      <c r="V10" s="20"/>
+      <c r="W10" s="20"/>
+      <c r="X10" s="20"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AA10" s="19"/>
+      <c r="AB10" s="19"/>
+      <c r="AC10" s="21"/>
+      <c r="AD10" s="19"/>
+      <c r="AE10" s="19"/>
+      <c r="AF10" s="19"/>
+      <c r="AH10" s="19"/>
+      <c r="AI10" s="19"/>
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="19"/>
+      <c r="AL10" s="21"/>
+      <c r="AM10" s="19"/>
+      <c r="AN10" s="19"/>
+      <c r="AO10" s="19"/>
+      <c r="AP10" s="19"/>
+      <c r="AQ10" s="19"/>
+      <c r="AR10" s="19"/>
+    </row>
+    <row r="11" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="19"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
+      <c r="T11" s="20"/>
+      <c r="U11" s="20"/>
+      <c r="V11" s="20"/>
+      <c r="W11" s="20"/>
+      <c r="X11" s="20"/>
+      <c r="Y11" s="19"/>
+      <c r="Z11" s="19"/>
+      <c r="AA11" s="19"/>
+      <c r="AB11" s="19"/>
+      <c r="AC11" s="21"/>
+      <c r="AD11" s="19"/>
+      <c r="AE11" s="19"/>
+      <c r="AF11" s="19"/>
+      <c r="AH11" s="19"/>
+      <c r="AI11" s="19"/>
+      <c r="AJ11" s="19"/>
+      <c r="AK11" s="19"/>
+      <c r="AL11" s="21"/>
+      <c r="AM11" s="19"/>
+      <c r="AN11" s="19"/>
+      <c r="AO11" s="19"/>
+      <c r="AP11" s="19"/>
+      <c r="AQ11" s="19"/>
+      <c r="AR11" s="19"/>
+    </row>
+    <row r="12" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="19"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="20"/>
+      <c r="S12" s="20"/>
+      <c r="T12" s="20"/>
+      <c r="U12" s="20"/>
+      <c r="V12" s="20"/>
+      <c r="W12" s="20"/>
+      <c r="X12" s="20"/>
+      <c r="Y12" s="19"/>
+      <c r="Z12" s="19"/>
+      <c r="AA12" s="19"/>
+      <c r="AB12" s="19"/>
+      <c r="AC12" s="21"/>
+      <c r="AD12" s="19"/>
+      <c r="AE12" s="19"/>
+      <c r="AF12" s="19"/>
+      <c r="AH12" s="19"/>
+      <c r="AI12" s="19"/>
+      <c r="AJ12" s="19"/>
+      <c r="AK12" s="19"/>
+      <c r="AL12" s="21"/>
+      <c r="AM12" s="19"/>
+      <c r="AN12" s="19"/>
+      <c r="AO12" s="19"/>
+      <c r="AP12" s="19"/>
+      <c r="AQ12" s="19"/>
+      <c r="AR12" s="19"/>
+    </row>
+    <row r="13" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="19"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="20"/>
+      <c r="P13" s="20"/>
+      <c r="Q13" s="20"/>
+      <c r="R13" s="20"/>
+      <c r="S13" s="20"/>
+      <c r="T13" s="20"/>
+      <c r="U13" s="20"/>
+      <c r="V13" s="20"/>
+      <c r="W13" s="20"/>
+      <c r="X13" s="20"/>
+      <c r="Y13" s="19"/>
+      <c r="Z13" s="19"/>
+      <c r="AA13" s="19"/>
+      <c r="AB13" s="19"/>
+      <c r="AC13" s="21"/>
+      <c r="AD13" s="19"/>
+      <c r="AE13" s="19"/>
+      <c r="AF13" s="19"/>
+      <c r="AH13" s="19"/>
+      <c r="AI13" s="19"/>
+      <c r="AJ13" s="19"/>
+      <c r="AK13" s="19"/>
+      <c r="AL13" s="21"/>
+      <c r="AM13" s="19"/>
+      <c r="AN13" s="19"/>
+      <c r="AO13" s="19"/>
+      <c r="AP13" s="19"/>
+      <c r="AQ13" s="19"/>
+      <c r="AR13" s="19"/>
+    </row>
+    <row r="14" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="19"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="20"/>
+      <c r="N14" s="20"/>
+      <c r="O14" s="20"/>
+      <c r="P14" s="20"/>
+      <c r="Q14" s="20"/>
+      <c r="R14" s="20"/>
+      <c r="S14" s="20"/>
+      <c r="T14" s="20"/>
+      <c r="U14" s="20"/>
+      <c r="V14" s="20"/>
+      <c r="W14" s="20"/>
+      <c r="X14" s="20"/>
+      <c r="Y14" s="19"/>
+      <c r="Z14" s="19"/>
+      <c r="AA14" s="19"/>
+      <c r="AB14" s="19"/>
+      <c r="AC14" s="21"/>
+      <c r="AD14" s="19"/>
+      <c r="AE14" s="19"/>
+      <c r="AF14" s="19"/>
+      <c r="AH14" s="19"/>
+      <c r="AI14" s="19"/>
+      <c r="AJ14" s="19"/>
+      <c r="AK14" s="19"/>
+      <c r="AL14" s="21"/>
+      <c r="AM14" s="19"/>
+      <c r="AN14" s="19"/>
+      <c r="AO14" s="19"/>
+      <c r="AP14" s="19"/>
+      <c r="AQ14" s="19"/>
+      <c r="AR14" s="19"/>
+    </row>
+    <row r="15" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="19"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="20"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="20"/>
+      <c r="S15" s="20"/>
+      <c r="T15" s="20"/>
+      <c r="U15" s="20"/>
+      <c r="V15" s="20"/>
+      <c r="W15" s="20"/>
+      <c r="X15" s="20"/>
+      <c r="Y15" s="19"/>
+      <c r="Z15" s="19"/>
+      <c r="AA15" s="19"/>
+      <c r="AB15" s="19"/>
+      <c r="AC15" s="21"/>
+      <c r="AD15" s="19"/>
+      <c r="AE15" s="19"/>
+      <c r="AF15" s="19"/>
+      <c r="AH15" s="19"/>
+      <c r="AI15" s="19"/>
+      <c r="AJ15" s="19"/>
+      <c r="AK15" s="19"/>
+      <c r="AL15" s="21"/>
+      <c r="AM15" s="19"/>
+      <c r="AN15" s="19"/>
+      <c r="AO15" s="19"/>
+      <c r="AP15" s="19"/>
+      <c r="AQ15" s="19"/>
+      <c r="AR15" s="19"/>
+    </row>
+    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="C16" s="15"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="15"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C18" s="15"/>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="15"/>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="15"/>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="15"/>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="15"/>
+    </row>
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="15"/>
+    </row>
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="15"/>
+    </row>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C25" s="15"/>
+    </row>
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C26" s="15"/>
+    </row>
+    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C27" s="15"/>
+    </row>
+    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C28" s="15"/>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="15"/>
+    </row>
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C30" s="15"/>
+    </row>
+    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C31" s="15"/>
+    </row>
+    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C32" s="15"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1228,6 +1871,241 @@
     <mergeCell ref="T1:X1"/>
     <mergeCell ref="AK1:AR1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:L15 S3:S15" xr:uid="{2F95256E-81D6-473E-9BA3-007ACDF1704C}">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1048576 O1:O1048576 P1:P1048576 Q1:Q1048576 R1:R1048576 T1:T1048576 U1:U1048576 V1:V1048576 W1:W1048576 X1:X1048576" xr:uid="{8567F238-0547-4193-A36E-6CA8E2EAE6B4}">
+      <formula1>"Sim,&lt;IGNORE&gt;"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Interno | Propriedade de Grupo HDI</oddFooter>
+  </headerFooter>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A7F1821A-C858-44B5-873C-A9A2945BD4D8}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$A$2:$A$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>A3:A15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{32A5A264-A84F-4761-9510-2CBC245B8C5D}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$B$2:$B$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>E3:E15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EBD8926B-0F74-4E96-A19D-4E90EBADFC50}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$C$2:$C$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>F3:F15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2C0CE9CB-D387-4195-B2B8-645D7ADBB7A4}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$D$2</xm:f>
+          </x14:formula1>
+          <xm:sqref>G3:G15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{76310054-FBC7-4DC4-A739-2340038BB9F2}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$E$2:$E$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>H3:H15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56168B89-78DD-43CE-A822-82F90EC2DBB0}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$F$2:$F$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>J3:J15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DF420454-E215-4342-A15C-8D2B3AD4E8EA}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$G$2:$G$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>M3:M15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D70141A0-4026-4172-A965-7EAAB28C6BEC}">
+          <x14:formula1>
+            <xm:f>Auxiliar!$H$2:$H$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>AC3:AC15</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72DDB486-0991-4A18-A792-EECA877FFCA3}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="59.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>79</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Interno | Propriedade de Grupo HDI</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{84698bb0-714d-4b99-b788-9371319a76a2}" enabled="1" method="Standard" siteId="{ccc49165-da44-4213-b797-fb01867c9d18}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Templates novos com bloco de proposta e template_proposta.xlsx
Scripts Python leem, preenchem, validam e corrigem o bloco opcional
"proposta" (listas do template) e o ramo "proposta" (só a proposta).
nucleo.js com a mesma mudança, ainda sem o teste de paridade; página e
documentação ainda não atualizadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETeciituSBa5wphWUasW8C
</commit_message>
<xml_diff>
--- a/.claude/skills/gerador-massas-seguros/templates/template_condominio_amplo.xlsx
+++ b/.claude/skills/gerador-massas-seguros/templates/template_condominio_amplo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb35177745223ee1/Área de Trabalho/TEMPLATES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{85FCB343-C9DD-4353-81A7-D8F49E45ACB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DD1C27E-6F33-48C3-A62E-D1292AF8AF75}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{85FCB343-C9DD-4353-81A7-D8F49E45ACB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0560C49F-699C-4B98-A1A1-185614C7056F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D1778361-77A0-49C1-A6FF-9F11D3ACD25C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="111">
   <si>
     <t>Dados CORRETOR</t>
   </si>
@@ -289,6 +289,90 @@
   </si>
   <si>
     <t>&lt;IGNORE&gt;</t>
+  </si>
+  <si>
+    <t>Endereço proponente</t>
+  </si>
+  <si>
+    <t>Contato proponente</t>
+  </si>
+  <si>
+    <t>Dados de Pagamento - Geral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debito </t>
+  </si>
+  <si>
+    <t>Proponente - CEP</t>
+  </si>
+  <si>
+    <t>Endereco Proponente - Número</t>
+  </si>
+  <si>
+    <t>Contato - Tipo Telefone</t>
+  </si>
+  <si>
+    <t>Contato - Telefone</t>
+  </si>
+  <si>
+    <t>Contato - Email</t>
+  </si>
+  <si>
+    <t>Proposta - Forma Pagamento</t>
+  </si>
+  <si>
+    <t>Proposta - Quantidade Parcelas</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Proponente Titular</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Documento Titular</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Nome Titular</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Banco</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Agência</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Dígito Agência</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Conta</t>
+  </si>
+  <si>
+    <t>Proposta Débito - Dígito Conta</t>
+  </si>
+  <si>
+    <t>Celular</t>
+  </si>
+  <si>
+    <t>Carnê</t>
+  </si>
+  <si>
+    <t>1 + 1</t>
+  </si>
+  <si>
+    <t>Residencial</t>
+  </si>
+  <si>
+    <t>Débito</t>
+  </si>
+  <si>
+    <t>1 + 2</t>
+  </si>
+  <si>
+    <t>Comercial</t>
+  </si>
+  <si>
+    <t>Cartão de Crédito</t>
+  </si>
+  <si>
+    <t>0 + 1</t>
   </si>
 </sst>
 </file>
@@ -369,7 +453,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -455,7 +539,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -527,7 +635,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -558,9 +666,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -576,7 +681,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -593,6 +699,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -934,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DB94AD-DD93-48A3-87B2-8FB065BB5A7F}">
-  <dimension ref="A1:AY33"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -980,9 +1094,23 @@
     <col min="42" max="42" width="34" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="34.85546875" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="29" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="17" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="30" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="23" t="s">
         <v>0</v>
@@ -1049,15 +1177,31 @@
       <c r="AP1" s="28"/>
       <c r="AQ1" s="28"/>
       <c r="AR1" s="28"/>
-      <c r="AS1" s="22"/>
-      <c r="AT1" s="22"/>
-      <c r="AU1" s="22"/>
-      <c r="AV1" s="22"/>
-      <c r="AW1" s="22"/>
-      <c r="AX1" s="22"/>
-      <c r="AY1" s="22"/>
-    </row>
-    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="AS1" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="AT1" s="29"/>
+      <c r="AU1" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="AV1" s="31"/>
+      <c r="AW1" s="31"/>
+      <c r="AX1" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY1" s="32"/>
+      <c r="AZ1" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="BA1" s="22"/>
+      <c r="BB1" s="22"/>
+      <c r="BC1" s="22"/>
+      <c r="BD1" s="22"/>
+      <c r="BE1" s="22"/>
+      <c r="BF1" s="22"/>
+      <c r="BG1" s="22"/>
+    </row>
+    <row r="2" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>11</v>
       </c>
@@ -1190,22 +1334,63 @@
       <c r="AR2" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="AS2" s="14"/>
-      <c r="AT2" s="14"/>
-      <c r="AU2" s="14"/>
-      <c r="AV2" s="14"/>
-    </row>
-    <row r="3" spans="1:51" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS2" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="AT2" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="AU2" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="AV2" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="AW2" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="AX2" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="AY2" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="AZ2" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA2" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="BB2" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="BC2" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="BD2" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="BE2" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="BF2" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="BG2" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:59" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="14">
         <v>72066486000171</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="15">
         <v>8040770</v>
       </c>
       <c r="E3" t="s">
@@ -1220,656 +1405,692 @@
       <c r="H3" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="I3" s="19">
+      <c r="I3" s="18">
         <v>1000000</v>
       </c>
       <c r="J3" t="s">
         <v>78</v>
       </c>
-      <c r="K3" s="20" t="s">
+      <c r="K3" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="L3" s="20" t="s">
+      <c r="L3" s="19" t="s">
         <v>78</v>
       </c>
       <c r="M3">
         <v>3</v>
       </c>
-      <c r="N3" s="20" t="s">
+      <c r="N3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="O3" s="20" t="s">
+      <c r="O3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="P3" s="20" t="s">
+      <c r="P3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="Q3" s="20" t="s">
+      <c r="Q3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="R3" s="20" t="s">
+      <c r="R3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="S3" s="20" t="s">
+      <c r="S3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="T3" s="20" t="s">
+      <c r="T3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="U3" s="20" t="s">
+      <c r="U3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="V3" s="20" t="s">
+      <c r="V3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="W3" s="20" t="s">
+      <c r="W3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="X3" s="20" t="s">
+      <c r="X3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="Y3" s="19">
+      <c r="Y3" s="18">
         <v>50000</v>
       </c>
-      <c r="Z3" s="19">
+      <c r="Z3" s="18">
         <v>35000</v>
       </c>
-      <c r="AA3" s="19">
+      <c r="AA3" s="18">
         <v>75000</v>
       </c>
-      <c r="AB3" s="19">
+      <c r="AB3" s="18">
         <v>35000</v>
       </c>
-      <c r="AC3" s="21">
+      <c r="AC3" s="20">
         <v>6</v>
       </c>
-      <c r="AD3" s="19">
+      <c r="AD3" s="18">
         <v>10000</v>
       </c>
-      <c r="AE3" s="19">
+      <c r="AE3" s="18">
         <v>10000</v>
       </c>
-      <c r="AF3" s="19">
+      <c r="AF3" s="18">
         <v>20000</v>
       </c>
       <c r="AG3" t="s">
         <v>82</v>
       </c>
-      <c r="AH3" s="19">
+      <c r="AH3" s="18">
         <v>20000</v>
       </c>
-      <c r="AI3" s="19">
+      <c r="AI3" s="18">
         <v>3000</v>
       </c>
-      <c r="AJ3" s="19">
+      <c r="AJ3" s="18">
         <v>35000</v>
       </c>
-      <c r="AK3" s="19">
+      <c r="AK3" s="18">
         <v>5000</v>
       </c>
-      <c r="AL3" s="21">
+      <c r="AL3" s="20">
         <v>10</v>
       </c>
-      <c r="AM3" s="19">
+      <c r="AM3" s="18">
         <v>5000</v>
       </c>
-      <c r="AN3" s="19">
+      <c r="AN3" s="18">
         <v>5000</v>
       </c>
-      <c r="AO3" s="19">
+      <c r="AO3" s="18">
         <v>5000</v>
       </c>
-      <c r="AP3" s="19">
+      <c r="AP3" s="18">
         <v>1000</v>
       </c>
-      <c r="AQ3" s="19"/>
-      <c r="AR3" s="19">
+      <c r="AQ3" s="18"/>
+      <c r="AR3" s="18">
         <v>3000</v>
       </c>
-    </row>
-    <row r="4" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="15"/>
-      <c r="D4" s="16"/>
+      <c r="AU3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>104</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:59" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
-      <c r="I4" s="19"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
-      <c r="Y4" s="19"/>
-      <c r="Z4" s="19"/>
-      <c r="AA4" s="19"/>
-      <c r="AB4" s="19"/>
-      <c r="AC4" s="21"/>
-      <c r="AD4" s="19"/>
-      <c r="AE4" s="19"/>
-      <c r="AF4" s="19"/>
-      <c r="AG4" s="19"/>
-      <c r="AH4" s="19"/>
-      <c r="AI4" s="19"/>
-      <c r="AJ4" s="19"/>
-      <c r="AK4" s="19"/>
-      <c r="AL4" s="21"/>
-      <c r="AM4" s="19"/>
-      <c r="AN4" s="19"/>
-      <c r="AO4" s="19"/>
-      <c r="AP4" s="19"/>
-      <c r="AQ4" s="19"/>
-      <c r="AR4" s="19"/>
-    </row>
-    <row r="5" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C5" s="15"/>
-      <c r="D5" s="16"/>
+      <c r="I4" s="18"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
+      <c r="Y4" s="18"/>
+      <c r="Z4" s="18"/>
+      <c r="AA4" s="18"/>
+      <c r="AB4" s="18"/>
+      <c r="AC4" s="20"/>
+      <c r="AD4" s="18"/>
+      <c r="AE4" s="18"/>
+      <c r="AF4" s="18"/>
+      <c r="AG4" s="18"/>
+      <c r="AH4" s="18"/>
+      <c r="AI4" s="18"/>
+      <c r="AJ4" s="18"/>
+      <c r="AK4" s="18"/>
+      <c r="AL4" s="20"/>
+      <c r="AM4" s="18"/>
+      <c r="AN4" s="18"/>
+      <c r="AO4" s="18"/>
+      <c r="AP4" s="18"/>
+      <c r="AQ4" s="18"/>
+      <c r="AR4" s="18"/>
+      <c r="AU4" t="s">
+        <v>105</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>106</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>107</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C5" s="14"/>
+      <c r="D5" s="15"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
-      <c r="I5" s="19"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20"/>
-      <c r="T5" s="20"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20"/>
-      <c r="Y5" s="19"/>
-      <c r="Z5" s="19"/>
-      <c r="AA5" s="19"/>
-      <c r="AB5" s="19"/>
-      <c r="AC5" s="21"/>
-      <c r="AD5" s="19"/>
-      <c r="AE5" s="19"/>
-      <c r="AF5" s="19"/>
-      <c r="AH5" s="19"/>
-      <c r="AI5" s="19"/>
-      <c r="AJ5" s="19"/>
-      <c r="AK5" s="19"/>
-      <c r="AL5" s="21"/>
-      <c r="AM5" s="19"/>
-      <c r="AN5" s="19"/>
-      <c r="AO5" s="19"/>
-      <c r="AP5" s="19"/>
-      <c r="AQ5" s="19"/>
-      <c r="AR5" s="19"/>
-    </row>
-    <row r="6" spans="1:51" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
+      <c r="I5" s="18"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="18"/>
+      <c r="AA5" s="18"/>
+      <c r="AB5" s="18"/>
+      <c r="AC5" s="20"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="18"/>
+      <c r="AF5" s="18"/>
+      <c r="AH5" s="18"/>
+      <c r="AI5" s="18"/>
+      <c r="AJ5" s="18"/>
+      <c r="AK5" s="18"/>
+      <c r="AL5" s="20"/>
+      <c r="AM5" s="18"/>
+      <c r="AN5" s="18"/>
+      <c r="AO5" s="18"/>
+      <c r="AP5" s="18"/>
+      <c r="AQ5" s="18"/>
+      <c r="AR5" s="18"/>
+      <c r="AU5" t="s">
+        <v>108</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>109</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:59" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="14"/>
+      <c r="D6" s="15"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
-      <c r="I6" s="19"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
-      <c r="T6" s="20"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
-      <c r="Y6" s="19"/>
-      <c r="Z6" s="19"/>
-      <c r="AA6" s="19"/>
-      <c r="AB6" s="19"/>
-      <c r="AC6" s="21"/>
-      <c r="AD6" s="19"/>
-      <c r="AE6" s="19"/>
-      <c r="AF6" s="19"/>
-      <c r="AH6" s="19"/>
-      <c r="AI6" s="19"/>
-      <c r="AJ6" s="19"/>
-      <c r="AK6" s="19"/>
-      <c r="AL6" s="21"/>
-      <c r="AM6" s="19"/>
-      <c r="AN6" s="19"/>
-      <c r="AO6" s="19"/>
-      <c r="AP6" s="19"/>
-      <c r="AQ6" s="19"/>
-      <c r="AR6" s="19"/>
-    </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
+      <c r="I6" s="18"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="18"/>
+      <c r="AA6" s="18"/>
+      <c r="AB6" s="18"/>
+      <c r="AC6" s="20"/>
+      <c r="AD6" s="18"/>
+      <c r="AE6" s="18"/>
+      <c r="AF6" s="18"/>
+      <c r="AH6" s="18"/>
+      <c r="AI6" s="18"/>
+      <c r="AJ6" s="18"/>
+      <c r="AK6" s="18"/>
+      <c r="AL6" s="20"/>
+      <c r="AM6" s="18"/>
+      <c r="AN6" s="18"/>
+      <c r="AO6" s="18"/>
+      <c r="AP6" s="18"/>
+      <c r="AQ6" s="18"/>
+      <c r="AR6" s="18"/>
+    </row>
+    <row r="7" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
-      <c r="I7" s="19"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="20"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="20"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="20"/>
-      <c r="Y7" s="19"/>
-      <c r="Z7" s="19"/>
-      <c r="AA7" s="19"/>
-      <c r="AB7" s="19"/>
-      <c r="AC7" s="21"/>
-      <c r="AD7" s="19"/>
-      <c r="AE7" s="19"/>
-      <c r="AF7" s="19"/>
-      <c r="AH7" s="19"/>
-      <c r="AI7" s="19"/>
-      <c r="AJ7" s="19"/>
-      <c r="AK7" s="19"/>
-      <c r="AL7" s="21"/>
-      <c r="AM7" s="19"/>
-      <c r="AN7" s="19"/>
-      <c r="AO7" s="19"/>
-      <c r="AP7" s="19"/>
-      <c r="AQ7" s="19"/>
-      <c r="AR7" s="19"/>
-    </row>
-    <row r="8" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
+      <c r="I7" s="18"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
+      <c r="Y7" s="18"/>
+      <c r="Z7" s="18"/>
+      <c r="AA7" s="18"/>
+      <c r="AB7" s="18"/>
+      <c r="AC7" s="20"/>
+      <c r="AD7" s="18"/>
+      <c r="AE7" s="18"/>
+      <c r="AF7" s="18"/>
+      <c r="AH7" s="18"/>
+      <c r="AI7" s="18"/>
+      <c r="AJ7" s="18"/>
+      <c r="AK7" s="18"/>
+      <c r="AL7" s="20"/>
+      <c r="AM7" s="18"/>
+      <c r="AN7" s="18"/>
+      <c r="AO7" s="18"/>
+      <c r="AP7" s="18"/>
+      <c r="AQ7" s="18"/>
+      <c r="AR7" s="18"/>
+    </row>
+    <row r="8" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C8" s="14"/>
+      <c r="D8" s="15"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-      <c r="I8" s="19"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-      <c r="T8" s="20"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20"/>
-      <c r="Y8" s="19"/>
-      <c r="Z8" s="19"/>
-      <c r="AA8" s="19"/>
-      <c r="AB8" s="19"/>
-      <c r="AC8" s="21"/>
-      <c r="AD8" s="19"/>
-      <c r="AE8" s="19"/>
-      <c r="AF8" s="19"/>
-      <c r="AH8" s="19"/>
-      <c r="AI8" s="19"/>
-      <c r="AJ8" s="19"/>
-      <c r="AK8" s="19"/>
-      <c r="AL8" s="21"/>
-      <c r="AM8" s="19"/>
-      <c r="AN8" s="19"/>
-      <c r="AO8" s="19"/>
-      <c r="AP8" s="19"/>
-      <c r="AQ8" s="19"/>
-      <c r="AR8" s="19"/>
-    </row>
-    <row r="9" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
+      <c r="I8" s="18"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
+      <c r="Y8" s="18"/>
+      <c r="Z8" s="18"/>
+      <c r="AA8" s="18"/>
+      <c r="AB8" s="18"/>
+      <c r="AC8" s="20"/>
+      <c r="AD8" s="18"/>
+      <c r="AE8" s="18"/>
+      <c r="AF8" s="18"/>
+      <c r="AH8" s="18"/>
+      <c r="AI8" s="18"/>
+      <c r="AJ8" s="18"/>
+      <c r="AK8" s="18"/>
+      <c r="AL8" s="20"/>
+      <c r="AM8" s="18"/>
+      <c r="AN8" s="18"/>
+      <c r="AO8" s="18"/>
+      <c r="AP8" s="18"/>
+      <c r="AQ8" s="18"/>
+      <c r="AR8" s="18"/>
+    </row>
+    <row r="9" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C9" s="14"/>
+      <c r="D9" s="15"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
-      <c r="I9" s="19"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
-      <c r="T9" s="20"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20"/>
-      <c r="Y9" s="19"/>
-      <c r="Z9" s="19"/>
-      <c r="AA9" s="19"/>
-      <c r="AB9" s="19"/>
-      <c r="AC9" s="21"/>
-      <c r="AD9" s="19"/>
-      <c r="AE9" s="19"/>
-      <c r="AF9" s="19"/>
-      <c r="AH9" s="19"/>
-      <c r="AI9" s="19"/>
-      <c r="AJ9" s="19"/>
-      <c r="AK9" s="19"/>
-      <c r="AL9" s="21"/>
-      <c r="AM9" s="19"/>
-      <c r="AN9" s="19"/>
-      <c r="AO9" s="19"/>
-      <c r="AP9" s="19"/>
-      <c r="AQ9" s="19"/>
-      <c r="AR9" s="19"/>
-    </row>
-    <row r="10" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
+      <c r="I9" s="18"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="18"/>
+      <c r="AC9" s="20"/>
+      <c r="AD9" s="18"/>
+      <c r="AE9" s="18"/>
+      <c r="AF9" s="18"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="18"/>
+      <c r="AJ9" s="18"/>
+      <c r="AK9" s="18"/>
+      <c r="AL9" s="20"/>
+      <c r="AM9" s="18"/>
+      <c r="AN9" s="18"/>
+      <c r="AO9" s="18"/>
+      <c r="AP9" s="18"/>
+      <c r="AQ9" s="18"/>
+      <c r="AR9" s="18"/>
+    </row>
+    <row r="10" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C10" s="14"/>
+      <c r="D10" s="15"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
-      <c r="I10" s="19"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-      <c r="N10" s="20"/>
-      <c r="O10" s="20"/>
-      <c r="P10" s="20"/>
-      <c r="Q10" s="20"/>
-      <c r="R10" s="20"/>
-      <c r="S10" s="20"/>
-      <c r="T10" s="20"/>
-      <c r="U10" s="20"/>
-      <c r="V10" s="20"/>
-      <c r="W10" s="20"/>
-      <c r="X10" s="20"/>
-      <c r="Y10" s="19"/>
-      <c r="Z10" s="19"/>
-      <c r="AA10" s="19"/>
-      <c r="AB10" s="19"/>
-      <c r="AC10" s="21"/>
-      <c r="AD10" s="19"/>
-      <c r="AE10" s="19"/>
-      <c r="AF10" s="19"/>
-      <c r="AH10" s="19"/>
-      <c r="AI10" s="19"/>
-      <c r="AJ10" s="19"/>
-      <c r="AK10" s="19"/>
-      <c r="AL10" s="21"/>
-      <c r="AM10" s="19"/>
-      <c r="AN10" s="19"/>
-      <c r="AO10" s="19"/>
-      <c r="AP10" s="19"/>
-      <c r="AQ10" s="19"/>
-      <c r="AR10" s="19"/>
-    </row>
-    <row r="11" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
+      <c r="I10" s="18"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
+      <c r="X10" s="19"/>
+      <c r="Y10" s="18"/>
+      <c r="Z10" s="18"/>
+      <c r="AA10" s="18"/>
+      <c r="AB10" s="18"/>
+      <c r="AC10" s="20"/>
+      <c r="AD10" s="18"/>
+      <c r="AE10" s="18"/>
+      <c r="AF10" s="18"/>
+      <c r="AH10" s="18"/>
+      <c r="AI10" s="18"/>
+      <c r="AJ10" s="18"/>
+      <c r="AK10" s="18"/>
+      <c r="AL10" s="20"/>
+      <c r="AM10" s="18"/>
+      <c r="AN10" s="18"/>
+      <c r="AO10" s="18"/>
+      <c r="AP10" s="18"/>
+      <c r="AQ10" s="18"/>
+      <c r="AR10" s="18"/>
+    </row>
+    <row r="11" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C11" s="14"/>
+      <c r="D11" s="15"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
-      <c r="I11" s="19"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="20"/>
-      <c r="P11" s="20"/>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="20"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-      <c r="X11" s="20"/>
-      <c r="Y11" s="19"/>
-      <c r="Z11" s="19"/>
-      <c r="AA11" s="19"/>
-      <c r="AB11" s="19"/>
-      <c r="AC11" s="21"/>
-      <c r="AD11" s="19"/>
-      <c r="AE11" s="19"/>
-      <c r="AF11" s="19"/>
-      <c r="AH11" s="19"/>
-      <c r="AI11" s="19"/>
-      <c r="AJ11" s="19"/>
-      <c r="AK11" s="19"/>
-      <c r="AL11" s="21"/>
-      <c r="AM11" s="19"/>
-      <c r="AN11" s="19"/>
-      <c r="AO11" s="19"/>
-      <c r="AP11" s="19"/>
-      <c r="AQ11" s="19"/>
-      <c r="AR11" s="19"/>
-    </row>
-    <row r="12" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="I11" s="18"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="19"/>
+      <c r="T11" s="19"/>
+      <c r="U11" s="19"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="19"/>
+      <c r="X11" s="19"/>
+      <c r="Y11" s="18"/>
+      <c r="Z11" s="18"/>
+      <c r="AA11" s="18"/>
+      <c r="AB11" s="18"/>
+      <c r="AC11" s="20"/>
+      <c r="AD11" s="18"/>
+      <c r="AE11" s="18"/>
+      <c r="AF11" s="18"/>
+      <c r="AH11" s="18"/>
+      <c r="AI11" s="18"/>
+      <c r="AJ11" s="18"/>
+      <c r="AK11" s="18"/>
+      <c r="AL11" s="20"/>
+      <c r="AM11" s="18"/>
+      <c r="AN11" s="18"/>
+      <c r="AO11" s="18"/>
+      <c r="AP11" s="18"/>
+      <c r="AQ11" s="18"/>
+      <c r="AR11" s="18"/>
+    </row>
+    <row r="12" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C12" s="14"/>
+      <c r="D12" s="15"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
-      <c r="I12" s="19"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="20"/>
-      <c r="P12" s="20"/>
-      <c r="Q12" s="20"/>
-      <c r="R12" s="20"/>
-      <c r="S12" s="20"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20"/>
-      <c r="Y12" s="19"/>
-      <c r="Z12" s="19"/>
-      <c r="AA12" s="19"/>
-      <c r="AB12" s="19"/>
-      <c r="AC12" s="21"/>
-      <c r="AD12" s="19"/>
-      <c r="AE12" s="19"/>
-      <c r="AF12" s="19"/>
-      <c r="AH12" s="19"/>
-      <c r="AI12" s="19"/>
-      <c r="AJ12" s="19"/>
-      <c r="AK12" s="19"/>
-      <c r="AL12" s="21"/>
-      <c r="AM12" s="19"/>
-      <c r="AN12" s="19"/>
-      <c r="AO12" s="19"/>
-      <c r="AP12" s="19"/>
-      <c r="AQ12" s="19"/>
-      <c r="AR12" s="19"/>
-    </row>
-    <row r="13" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="I12" s="18"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="19"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19"/>
+      <c r="X12" s="19"/>
+      <c r="Y12" s="18"/>
+      <c r="Z12" s="18"/>
+      <c r="AA12" s="18"/>
+      <c r="AB12" s="18"/>
+      <c r="AC12" s="20"/>
+      <c r="AD12" s="18"/>
+      <c r="AE12" s="18"/>
+      <c r="AF12" s="18"/>
+      <c r="AH12" s="18"/>
+      <c r="AI12" s="18"/>
+      <c r="AJ12" s="18"/>
+      <c r="AK12" s="18"/>
+      <c r="AL12" s="20"/>
+      <c r="AM12" s="18"/>
+      <c r="AN12" s="18"/>
+      <c r="AO12" s="18"/>
+      <c r="AP12" s="18"/>
+      <c r="AQ12" s="18"/>
+      <c r="AR12" s="18"/>
+    </row>
+    <row r="13" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C13" s="14"/>
+      <c r="D13" s="15"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
-      <c r="I13" s="19"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="N13" s="20"/>
-      <c r="O13" s="20"/>
-      <c r="P13" s="20"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="20"/>
-      <c r="S13" s="20"/>
-      <c r="T13" s="20"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="20"/>
-      <c r="W13" s="20"/>
-      <c r="X13" s="20"/>
-      <c r="Y13" s="19"/>
-      <c r="Z13" s="19"/>
-      <c r="AA13" s="19"/>
-      <c r="AB13" s="19"/>
-      <c r="AC13" s="21"/>
-      <c r="AD13" s="19"/>
-      <c r="AE13" s="19"/>
-      <c r="AF13" s="19"/>
-      <c r="AH13" s="19"/>
-      <c r="AI13" s="19"/>
-      <c r="AJ13" s="19"/>
-      <c r="AK13" s="19"/>
-      <c r="AL13" s="21"/>
-      <c r="AM13" s="19"/>
-      <c r="AN13" s="19"/>
-      <c r="AO13" s="19"/>
-      <c r="AP13" s="19"/>
-      <c r="AQ13" s="19"/>
-      <c r="AR13" s="19"/>
-    </row>
-    <row r="14" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
+      <c r="I13" s="18"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="19"/>
+      <c r="Q13" s="19"/>
+      <c r="R13" s="19"/>
+      <c r="S13" s="19"/>
+      <c r="T13" s="19"/>
+      <c r="U13" s="19"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="19"/>
+      <c r="X13" s="19"/>
+      <c r="Y13" s="18"/>
+      <c r="Z13" s="18"/>
+      <c r="AA13" s="18"/>
+      <c r="AB13" s="18"/>
+      <c r="AC13" s="20"/>
+      <c r="AD13" s="18"/>
+      <c r="AE13" s="18"/>
+      <c r="AF13" s="18"/>
+      <c r="AH13" s="18"/>
+      <c r="AI13" s="18"/>
+      <c r="AJ13" s="18"/>
+      <c r="AK13" s="18"/>
+      <c r="AL13" s="20"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="18"/>
+      <c r="AO13" s="18"/>
+      <c r="AP13" s="18"/>
+      <c r="AQ13" s="18"/>
+      <c r="AR13" s="18"/>
+    </row>
+    <row r="14" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
-      <c r="I14" s="19"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="N14" s="20"/>
-      <c r="O14" s="20"/>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="20"/>
-      <c r="S14" s="20"/>
-      <c r="T14" s="20"/>
-      <c r="U14" s="20"/>
-      <c r="V14" s="20"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="20"/>
-      <c r="Y14" s="19"/>
-      <c r="Z14" s="19"/>
-      <c r="AA14" s="19"/>
-      <c r="AB14" s="19"/>
-      <c r="AC14" s="21"/>
-      <c r="AD14" s="19"/>
-      <c r="AE14" s="19"/>
-      <c r="AF14" s="19"/>
-      <c r="AH14" s="19"/>
-      <c r="AI14" s="19"/>
-      <c r="AJ14" s="19"/>
-      <c r="AK14" s="19"/>
-      <c r="AL14" s="21"/>
-      <c r="AM14" s="19"/>
-      <c r="AN14" s="19"/>
-      <c r="AO14" s="19"/>
-      <c r="AP14" s="19"/>
-      <c r="AQ14" s="19"/>
-      <c r="AR14" s="19"/>
-    </row>
-    <row r="15" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="I14" s="18"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19"/>
+      <c r="X14" s="19"/>
+      <c r="Y14" s="18"/>
+      <c r="Z14" s="18"/>
+      <c r="AA14" s="18"/>
+      <c r="AB14" s="18"/>
+      <c r="AC14" s="20"/>
+      <c r="AD14" s="18"/>
+      <c r="AE14" s="18"/>
+      <c r="AF14" s="18"/>
+      <c r="AH14" s="18"/>
+      <c r="AI14" s="18"/>
+      <c r="AJ14" s="18"/>
+      <c r="AK14" s="18"/>
+      <c r="AL14" s="20"/>
+      <c r="AM14" s="18"/>
+      <c r="AN14" s="18"/>
+      <c r="AO14" s="18"/>
+      <c r="AP14" s="18"/>
+      <c r="AQ14" s="18"/>
+      <c r="AR14" s="18"/>
+    </row>
+    <row r="15" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C15" s="14"/>
+      <c r="D15" s="15"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
-      <c r="I15" s="19"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="N15" s="20"/>
-      <c r="O15" s="20"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20"/>
-      <c r="T15" s="20"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="20"/>
-      <c r="Y15" s="19"/>
-      <c r="Z15" s="19"/>
-      <c r="AA15" s="19"/>
-      <c r="AB15" s="19"/>
-      <c r="AC15" s="21"/>
-      <c r="AD15" s="19"/>
-      <c r="AE15" s="19"/>
-      <c r="AF15" s="19"/>
-      <c r="AH15" s="19"/>
-      <c r="AI15" s="19"/>
-      <c r="AJ15" s="19"/>
-      <c r="AK15" s="19"/>
-      <c r="AL15" s="21"/>
-      <c r="AM15" s="19"/>
-      <c r="AN15" s="19"/>
-      <c r="AO15" s="19"/>
-      <c r="AP15" s="19"/>
-      <c r="AQ15" s="19"/>
-      <c r="AR15" s="19"/>
-    </row>
-    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="C16" s="15"/>
+      <c r="I15" s="18"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="19"/>
+      <c r="S15" s="19"/>
+      <c r="T15" s="19"/>
+      <c r="U15" s="19"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="19"/>
+      <c r="Y15" s="18"/>
+      <c r="Z15" s="18"/>
+      <c r="AA15" s="18"/>
+      <c r="AB15" s="18"/>
+      <c r="AC15" s="20"/>
+      <c r="AD15" s="18"/>
+      <c r="AE15" s="18"/>
+      <c r="AF15" s="18"/>
+      <c r="AH15" s="18"/>
+      <c r="AI15" s="18"/>
+      <c r="AJ15" s="18"/>
+      <c r="AK15" s="18"/>
+      <c r="AL15" s="20"/>
+      <c r="AM15" s="18"/>
+      <c r="AN15" s="18"/>
+      <c r="AO15" s="18"/>
+      <c r="AP15" s="18"/>
+      <c r="AQ15" s="18"/>
+      <c r="AR15" s="18"/>
+    </row>
+    <row r="16" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="C16" s="14"/>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="15"/>
+      <c r="C17" s="14"/>
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C18" s="15"/>
+      <c r="C18" s="14"/>
     </row>
     <row r="19" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C19" s="15"/>
+      <c r="C19" s="14"/>
     </row>
     <row r="20" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C20" s="15"/>
+      <c r="C20" s="14"/>
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C21" s="15"/>
+      <c r="C21" s="14"/>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C22" s="15"/>
+      <c r="C22" s="14"/>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="15"/>
+      <c r="C23" s="14"/>
     </row>
     <row r="24" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C24" s="15"/>
+      <c r="C24" s="14"/>
     </row>
     <row r="25" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="15"/>
+      <c r="C25" s="14"/>
     </row>
     <row r="26" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="15"/>
+      <c r="C26" s="14"/>
     </row>
     <row r="27" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C27" s="15"/>
+      <c r="C27" s="14"/>
     </row>
     <row r="28" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="15"/>
+      <c r="C28" s="14"/>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="15"/>
+      <c r="C29" s="14"/>
     </row>
     <row r="30" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C30" s="15"/>
+      <c r="C30" s="14"/>
     </row>
     <row r="31" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C31" s="15"/>
+      <c r="C31" s="14"/>
     </row>
     <row r="32" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C32" s="15"/>
+      <c r="C32" s="14"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="15"/>
+      <c r="C33" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="AS1:AY1"/>
+  <mergeCells count="9">
+    <mergeCell ref="AZ1:BG1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="N1:R1"/>
     <mergeCell ref="T1:X1"/>
     <mergeCell ref="AK1:AR1"/>
+    <mergeCell ref="AS1:AT1"/>
+    <mergeCell ref="AU1:AW1"/>
+    <mergeCell ref="AX1:AY1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:L15 S3:S15" xr:uid="{2F95256E-81D6-473E-9BA3-007ACDF1704C}">
@@ -1985,7 +2206,7 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>55</v>
       </c>
       <c r="C2" t="s">
@@ -1997,7 +2218,7 @@
       <c r="E2" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>78</v>
       </c>
       <c r="G2">
@@ -2011,7 +2232,7 @@
       <c r="A3" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>56</v>
       </c>
       <c r="C3" t="s">
@@ -2020,7 +2241,7 @@
       <c r="E3" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="17" t="s">
         <v>77</v>
       </c>
       <c r="G3">
@@ -2034,7 +2255,7 @@
       <c r="A4" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="16" t="s">
         <v>57</v>
       </c>
       <c r="C4" t="s">
@@ -2051,7 +2272,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>58</v>
       </c>
       <c r="G5">
@@ -2062,7 +2283,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="16" t="s">
         <v>59</v>
       </c>
       <c r="G6">
@@ -2073,7 +2294,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>60</v>
       </c>
       <c r="G7" t="s">
@@ -2084,7 +2305,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>61</v>
       </c>
       <c r="G8" t="s">
@@ -2092,7 +2313,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>